<commit_message>
Todos los enlaces internos ahora apuntan correctamente a 01-assessment-context.md considerando la nueva estructura de directorios.
</commit_message>
<xml_diff>
--- a/Grupo_Salinas_Checklist (IGS).xlsx
+++ b/Grupo_Salinas_Checklist (IGS).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cesar/Herd/IGS-Billing/docs/igs-mx-baz-biso/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1AC95EF7-3DC0-154B-8B6A-E20978474E6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63438EC5-0D55-A547-83BB-12346D311A22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3600" yWindow="2040" windowWidth="28360" windowHeight="16260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Hoja1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Terceros!$A$7:$J$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Terceros!$A$7:$K$42</definedName>
   </definedNames>
   <calcPr calcId="0"/>
   <extLst>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="185">
   <si>
     <t>DSI-CSF-CSA-</t>
   </si>
@@ -185,9 +185,6 @@
     <t>Mostrar las políticas de monitoreo así como evidencias del tipo de incidentes, alertas, etc. que generan</t>
   </si>
   <si>
-    <t>Medidas tecnicas y de control</t>
-  </si>
-  <si>
     <t>El proveedor deberá contar con políticas y procedimientos de respuestas a incidentes</t>
   </si>
   <si>
@@ -291,9 +288,6 @@
   </si>
   <si>
     <t>Mostrar evidencia de como realiza la autenticación de los usuarios</t>
-  </si>
-  <si>
-    <t>Se tiene establecido un modelo de Autenticación basado en roles y permisos. El usuario se loguea con mail verificado y su contraseña, y obtiene tokens de sesión que duran hasta 60 minutos y se desechan en automatico después de este tiempo. Adicional, los usuarios y roles criticos, requieren 2FA, antes de obtener el token</t>
   </si>
   <si>
     <t>La aplicación deberá contar con métodos de autorización de usuarios</t>
@@ -549,9 +543,6 @@
     <t>No presentan un diagrama de arquitectura donde tengan hospedada su solución.</t>
   </si>
   <si>
-    <t>No se entregó diagrama de la VPN con Grupo Salinas.</t>
-  </si>
-  <si>
     <t>El servicio se opera 100 % sobre AWS. Heredado de AWS (SOC 2 / ISO 27001 AWS).</t>
   </si>
   <si>
@@ -561,16 +552,10 @@
     <t>Cumple parcialmente.</t>
   </si>
   <si>
-    <t>Adjuntar una muestra de alertas SIEM reales.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Política vigente y declaración AES-256 en reposo. </t>
   </si>
   <si>
     <t>Acceso via API HTTPS / TLS 1.2.</t>
-  </si>
-  <si>
-    <t>IGS usa Bearer Token propio con 2FA, sesiones de 60 min. No hay SAML 2.0 ni OAuth 2.0 federado.</t>
   </si>
   <si>
     <t>Cumple, Parcialmente</t>
@@ -617,12 +602,33 @@
   <si>
     <t>Debe incluirse en el contrato con cláusulas claras de responsabilidad, penalizaciones y notificación</t>
   </si>
+  <si>
+    <t>En progreso.</t>
+  </si>
+  <si>
+    <t>No se cuenta aún con la IP pública de Grupo Salinas, por tanto no se ha configurado ni documentado la conectividad por VPN.</t>
+  </si>
+  <si>
+    <t>The solution currently includes application-layer monitoring, security logging, auditing, and production observability controls. Laravel Nightwatch is used for observability and error tracking; however, it is not relied upon as a substitute for a centralized SIEM platform. Therefore, the requirement is currently considered partially compliant pending centralized SIEM evidence and real alert samples from production operations.</t>
+  </si>
+  <si>
+    <t>https://github.com/IGS-Mexico-DEV/IGS-MX-BAZ-BISO/tree/main/Req.%2006</t>
+  </si>
+  <si>
+    <t>Se genera conforme a disponibilidad de información para generar la interface.</t>
+  </si>
+  <si>
+    <t>https://github.com/IGS-Mexico-DEV/IGS-MX-BAZ-BISO/tree/main/Req.%2014</t>
+  </si>
+  <si>
+    <t>The application currently implements user authentication through session-based web authentication, API token authentication, email verification, role-based access control, and OTP-based MFA for privileged users. These controls provide evidence of how user authentication is performed. However, no repository-verifiable evidence of federated access control through SAML 2.0 or OAuth 2.0 has been identified. Therefore, the requirement is currently considered partially compliant pending federation implementation evidence or external production evidence.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -667,8 +673,14 @@
       <color theme="0"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -714,6 +726,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -867,7 +885,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -908,13 +926,7 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -938,6 +950,25 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1193,6 +1224,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:V1000"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1238,15 +1270,15 @@
       <c r="C2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="19" t="s">
+      <c r="D2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
-      <c r="I2" s="21"/>
-      <c r="J2" s="22"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="20"/>
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
       <c r="M2" s="1"/>
@@ -1266,11 +1298,11 @@
       <c r="C3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="25" t="s">
+      <c r="D3" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="20"/>
-      <c r="F3" s="21"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="19"/>
       <c r="G3" s="4" t="s">
         <v>4</v>
       </c>
@@ -1280,7 +1312,7 @@
       <c r="I3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="J3" s="23"/>
+      <c r="J3" s="21"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
@@ -1300,15 +1332,15 @@
       <c r="C4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="25"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="21"/>
-      <c r="G4" s="26" t="s">
+      <c r="D4" s="23"/>
+      <c r="E4" s="18"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="H4" s="20"/>
-      <c r="I4" s="21"/>
-      <c r="J4" s="24"/>
+      <c r="H4" s="18"/>
+      <c r="I4" s="19"/>
+      <c r="J4" s="22"/>
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
       <c r="M4" s="1"/>
@@ -1402,7 +1434,7 @@
         <v>16</v>
       </c>
       <c r="K7" s="7" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
@@ -1438,13 +1470,13 @@
         <v>21</v>
       </c>
       <c r="I8" s="9" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="J8" s="9" t="s">
         <v>22</v>
       </c>
       <c r="K8" s="9" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
@@ -1458,76 +1490,76 @@
       <c r="U8" s="2"/>
       <c r="V8" s="2"/>
     </row>
-    <row r="9" spans="1:22" ht="80" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:22" s="29" customFormat="1" ht="80" x14ac:dyDescent="0.2">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
-      <c r="C9" s="9">
+      <c r="C9" s="25">
         <v>2</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="25" t="s">
         <v>23</v>
       </c>
       <c r="F9" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="G9" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="H9" s="9" t="s">
+      <c r="H9" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="I9" s="9" t="s">
-        <v>157</v>
-      </c>
-      <c r="J9" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="K9" s="9" t="s">
-        <v>160</v>
-      </c>
-      <c r="L9" s="1"/>
-      <c r="M9" s="1"/>
-      <c r="N9" s="1"/>
-      <c r="O9" s="1"/>
-      <c r="P9" s="1"/>
-      <c r="Q9" s="1"/>
-      <c r="R9" s="1"/>
-      <c r="S9" s="1"/>
-      <c r="T9" s="2"/>
-      <c r="U9" s="2"/>
-      <c r="V9" s="2"/>
-    </row>
-    <row r="10" spans="1:22" ht="80" x14ac:dyDescent="0.2">
+      <c r="I9" s="26" t="s">
+        <v>178</v>
+      </c>
+      <c r="J9" s="26" t="s">
+        <v>182</v>
+      </c>
+      <c r="K9" s="26" t="s">
+        <v>179</v>
+      </c>
+      <c r="L9" s="27"/>
+      <c r="M9" s="27"/>
+      <c r="N9" s="27"/>
+      <c r="O9" s="27"/>
+      <c r="P9" s="27"/>
+      <c r="Q9" s="27"/>
+      <c r="R9" s="27"/>
+      <c r="S9" s="27"/>
+      <c r="T9" s="28"/>
+      <c r="U9" s="28"/>
+      <c r="V9" s="28"/>
+    </row>
+    <row r="10" spans="1:22" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
-      <c r="C10" s="10">
+      <c r="C10" s="25">
         <v>3</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="E10" s="25" t="s">
         <v>27</v>
       </c>
       <c r="F10" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="G10" s="10" t="s">
+      <c r="G10" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="H10" s="10" t="s">
+      <c r="H10" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="I10" s="10" t="s">
+      <c r="I10" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="J10" s="10" t="s">
+      <c r="J10" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="K10" s="10" t="s">
+      <c r="K10" s="25" t="s">
         <v>26</v>
       </c>
       <c r="L10" s="1"/>
@@ -1542,35 +1574,35 @@
       <c r="U10" s="2"/>
       <c r="V10" s="2"/>
     </row>
-    <row r="11" spans="1:22" ht="48" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:22" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
-      <c r="C11" s="9">
+      <c r="C11" s="25">
         <v>4</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="E11" s="10" t="s">
+      <c r="E11" s="25" t="s">
         <v>31</v>
       </c>
       <c r="F11" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="G11" s="10" t="s">
+      <c r="G11" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="H11" s="10" t="s">
+      <c r="H11" s="25" t="s">
         <v>34</v>
       </c>
-      <c r="I11" s="10" t="s">
+      <c r="I11" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="J11" s="10" t="s">
+      <c r="J11" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="K11" s="10" t="s">
-        <v>161</v>
+      <c r="K11" s="25" t="s">
+        <v>158</v>
       </c>
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
@@ -1584,35 +1616,35 @@
       <c r="U11" s="2"/>
       <c r="V11" s="2"/>
     </row>
-    <row r="12" spans="1:22" ht="80" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:22" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12" s="11"/>
       <c r="B12" s="11"/>
-      <c r="C12" s="9">
+      <c r="C12" s="25">
         <v>5</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="E12" s="25" t="s">
         <v>36</v>
       </c>
       <c r="F12" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="G12" s="10" t="s">
+      <c r="G12" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="H12" s="10" t="s">
+      <c r="H12" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="I12" s="10" t="s">
+      <c r="I12" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="J12" s="10" t="s">
+      <c r="J12" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="K12" s="10" t="s">
-        <v>162</v>
+      <c r="K12" s="25" t="s">
+        <v>159</v>
       </c>
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
@@ -1626,76 +1658,76 @@
       <c r="U12" s="2"/>
       <c r="V12" s="2"/>
     </row>
-    <row r="13" spans="1:22" ht="138" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:22" s="29" customFormat="1" ht="138" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1"/>
       <c r="B13" s="12"/>
-      <c r="C13" s="13">
+      <c r="C13" s="25">
         <v>6</v>
       </c>
-      <c r="D13" s="13" t="s">
+      <c r="D13" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="E13" s="13" t="s">
+      <c r="E13" s="25" t="s">
         <v>37</v>
       </c>
       <c r="F13" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="G13" s="13" t="s">
+      <c r="G13" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="H13" s="13" t="s">
+      <c r="H13" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="I13" s="13" t="s">
-        <v>163</v>
-      </c>
-      <c r="J13" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="K13" s="13" t="s">
-        <v>164</v>
-      </c>
-      <c r="L13" s="1"/>
-      <c r="M13" s="1"/>
-      <c r="N13" s="1"/>
-      <c r="O13" s="1"/>
-      <c r="P13" s="1"/>
-      <c r="Q13" s="1"/>
-      <c r="R13" s="1"/>
-      <c r="S13" s="1"/>
-      <c r="T13" s="2"/>
-      <c r="U13" s="2"/>
-      <c r="V13" s="2"/>
-    </row>
-    <row r="14" spans="1:22" ht="80" x14ac:dyDescent="0.2">
+      <c r="I13" s="25" t="s">
+        <v>160</v>
+      </c>
+      <c r="J13" s="25" t="s">
+        <v>181</v>
+      </c>
+      <c r="K13" s="26" t="s">
+        <v>180</v>
+      </c>
+      <c r="L13" s="27"/>
+      <c r="M13" s="27"/>
+      <c r="N13" s="27"/>
+      <c r="O13" s="27"/>
+      <c r="P13" s="27"/>
+      <c r="Q13" s="27"/>
+      <c r="R13" s="27"/>
+      <c r="S13" s="27"/>
+      <c r="T13" s="28"/>
+      <c r="U13" s="28"/>
+      <c r="V13" s="28"/>
+    </row>
+    <row r="14" spans="1:22" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
-      <c r="C14" s="10">
+      <c r="C14" s="25">
         <v>7</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D14" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="E14" s="10" t="s">
-        <v>42</v>
+      <c r="E14" s="25" t="s">
+        <v>41</v>
       </c>
       <c r="F14" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="G14" s="10" t="s">
+      <c r="G14" s="25" t="s">
+        <v>42</v>
+      </c>
+      <c r="H14" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="H14" s="10" t="s">
+      <c r="I14" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="J14" s="25" t="s">
         <v>44</v>
       </c>
-      <c r="I14" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="J14" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="K14" s="10" t="s">
+      <c r="K14" s="25" t="s">
         <v>26</v>
       </c>
       <c r="L14" s="1"/>
@@ -1710,34 +1742,34 @@
       <c r="U14" s="2"/>
       <c r="V14" s="2"/>
     </row>
-    <row r="15" spans="1:22" ht="69" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:22" ht="69" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
-      <c r="C15" s="10">
+      <c r="C15" s="25">
         <v>8</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="E15" s="25" t="s">
+        <v>45</v>
+      </c>
+      <c r="F15" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="F15" s="10" t="s">
+      <c r="G15" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="G15" s="10" t="s">
+      <c r="H15" s="25" t="s">
         <v>48</v>
       </c>
-      <c r="H15" s="10" t="s">
+      <c r="I15" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="J15" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="I15" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="J15" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="K15" s="10" t="s">
+      <c r="K15" s="25" t="s">
         <v>26</v>
       </c>
       <c r="L15" s="1"/>
@@ -1752,34 +1784,34 @@
       <c r="U15" s="2"/>
       <c r="V15" s="2"/>
     </row>
-    <row r="16" spans="1:22" ht="106" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:22" ht="106" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
-      <c r="C16" s="10">
+      <c r="C16" s="25">
         <v>9</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="D16" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="E16" s="10" t="s">
+      <c r="E16" s="25" t="s">
+        <v>50</v>
+      </c>
+      <c r="F16" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="G16" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="F16" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="G16" s="10" t="s">
+      <c r="H16" s="25" t="s">
         <v>52</v>
       </c>
-      <c r="H16" s="10" t="s">
+      <c r="I16" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="J16" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="I16" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="J16" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="K16" s="10" t="s">
+      <c r="K16" s="25" t="s">
         <v>26</v>
       </c>
       <c r="L16" s="1"/>
@@ -1794,34 +1826,34 @@
       <c r="U16" s="2"/>
       <c r="V16" s="2"/>
     </row>
-    <row r="17" spans="1:22" ht="64" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:22" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1"/>
       <c r="B17" s="11"/>
-      <c r="C17" s="10">
+      <c r="C17" s="25">
         <v>10</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="D17" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="E17" s="10" t="s">
+      <c r="E17" s="25" t="s">
+        <v>54</v>
+      </c>
+      <c r="F17" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="G17" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="F17" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="G17" s="10" t="s">
+      <c r="H17" s="25" t="s">
         <v>56</v>
       </c>
-      <c r="H17" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="I17" s="10" t="s">
+      <c r="I17" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="J17" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="K17" s="10" t="s">
+      <c r="J17" s="25" t="s">
+        <v>49</v>
+      </c>
+      <c r="K17" s="25" t="s">
         <v>26</v>
       </c>
       <c r="L17" s="1"/>
@@ -1836,35 +1868,35 @@
       <c r="U17" s="2"/>
       <c r="V17" s="2"/>
     </row>
-    <row r="18" spans="1:22" ht="64" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:22" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
-      <c r="C18" s="10">
+      <c r="C18" s="25">
         <v>11</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="D18" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="E18" s="10" t="s">
+      <c r="E18" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="F18" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="F18" s="10" t="s">
+      <c r="G18" s="25" t="s">
         <v>59</v>
       </c>
-      <c r="G18" s="10" t="s">
+      <c r="H18" s="25" t="s">
         <v>60</v>
       </c>
-      <c r="H18" s="10" t="s">
+      <c r="I18" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="J18" s="25" t="s">
         <v>61</v>
       </c>
-      <c r="I18" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="J18" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="K18" s="10" t="s">
-        <v>165</v>
+      <c r="K18" s="25" t="s">
+        <v>161</v>
       </c>
       <c r="L18" s="1"/>
       <c r="M18" s="1"/>
@@ -1878,34 +1910,34 @@
       <c r="U18" s="2"/>
       <c r="V18" s="2"/>
     </row>
-    <row r="19" spans="1:22" ht="64" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:22" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
-      <c r="C19" s="10">
+      <c r="C19" s="25">
         <v>12</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="D19" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="E19" s="10" t="s">
+      <c r="E19" s="25" t="s">
+        <v>62</v>
+      </c>
+      <c r="F19" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="F19" s="10" t="s">
+      <c r="G19" s="25" t="s">
         <v>64</v>
       </c>
-      <c r="G19" s="10" t="s">
+      <c r="H19" s="25" t="s">
         <v>65</v>
       </c>
-      <c r="H19" s="10" t="s">
+      <c r="I19" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="J19" s="25" t="s">
         <v>66</v>
       </c>
-      <c r="I19" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="J19" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="K19" s="14" t="s">
+      <c r="K19" s="30" t="s">
         <v>26</v>
       </c>
       <c r="L19" s="1"/>
@@ -1920,35 +1952,35 @@
       <c r="U19" s="2"/>
       <c r="V19" s="2"/>
     </row>
-    <row r="20" spans="1:22" ht="48" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:22" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
-      <c r="C20" s="10">
+      <c r="C20" s="25">
         <v>13</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" s="25" t="s">
+        <v>67</v>
+      </c>
+      <c r="E20" s="25" t="s">
         <v>68</v>
       </c>
-      <c r="E20" s="10" t="s">
+      <c r="F20" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="G20" s="25" t="s">
         <v>69</v>
       </c>
-      <c r="F20" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="G20" s="10" t="s">
+      <c r="H20" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="H20" s="10" t="s">
+      <c r="I20" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="J20" s="25" t="s">
         <v>71</v>
       </c>
-      <c r="I20" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="J20" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="K20" s="11" t="s">
-        <v>166</v>
+      <c r="K20" s="27" t="s">
+        <v>162</v>
       </c>
       <c r="L20" s="1"/>
       <c r="M20" s="1"/>
@@ -1962,77 +1994,77 @@
       <c r="U20" s="2"/>
       <c r="V20" s="2"/>
     </row>
-    <row r="21" spans="1:22" ht="96" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:22" s="29" customFormat="1" ht="224" x14ac:dyDescent="0.2">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
-      <c r="C21" s="15">
+      <c r="C21" s="25">
         <v>14</v>
       </c>
-      <c r="D21" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="E21" s="15" t="s">
+      <c r="D21" s="25" t="s">
+        <v>67</v>
+      </c>
+      <c r="E21" s="25" t="s">
+        <v>72</v>
+      </c>
+      <c r="F21" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="F21" s="15" t="s">
+      <c r="G21" s="25" t="s">
         <v>74</v>
       </c>
-      <c r="G21" s="15" t="s">
+      <c r="H21" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="H21" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="I21" s="15" t="s">
-        <v>157</v>
-      </c>
-      <c r="J21" s="15" t="s">
-        <v>77</v>
-      </c>
-      <c r="K21" s="16" t="s">
-        <v>167</v>
-      </c>
-      <c r="L21" s="1"/>
-      <c r="M21" s="1"/>
-      <c r="N21" s="1"/>
-      <c r="O21" s="1"/>
-      <c r="P21" s="1"/>
-      <c r="Q21" s="1"/>
-      <c r="R21" s="1"/>
-      <c r="S21" s="1"/>
-      <c r="T21" s="2"/>
-      <c r="U21" s="2"/>
-      <c r="V21" s="2"/>
+      <c r="I21" s="26" t="s">
+        <v>160</v>
+      </c>
+      <c r="J21" s="25" t="s">
+        <v>183</v>
+      </c>
+      <c r="K21" s="31" t="s">
+        <v>184</v>
+      </c>
+      <c r="L21" s="27"/>
+      <c r="M21" s="27"/>
+      <c r="N21" s="27"/>
+      <c r="O21" s="27"/>
+      <c r="P21" s="27"/>
+      <c r="Q21" s="27"/>
+      <c r="R21" s="27"/>
+      <c r="S21" s="27"/>
+      <c r="T21" s="28"/>
+      <c r="U21" s="28"/>
+      <c r="V21" s="28"/>
     </row>
     <row r="22" spans="1:22" ht="59" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
-      <c r="C22" s="17">
+      <c r="C22" s="15">
         <v>15</v>
       </c>
-      <c r="D22" s="17" t="s">
-        <v>68</v>
-      </c>
-      <c r="E22" s="17" t="s">
+      <c r="D22" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="E22" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="F22" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="G22" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="H22" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="I22" s="15" t="s">
+        <v>163</v>
+      </c>
+      <c r="J22" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="F22" s="17" t="s">
-        <v>74</v>
-      </c>
-      <c r="G22" s="17" t="s">
-        <v>75</v>
-      </c>
-      <c r="H22" s="17" t="s">
-        <v>79</v>
-      </c>
-      <c r="I22" s="17" t="s">
-        <v>168</v>
-      </c>
-      <c r="J22" s="17" t="s">
-        <v>80</v>
-      </c>
       <c r="K22" s="13" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="L22" s="1"/>
       <c r="M22" s="1"/>
@@ -2049,32 +2081,32 @@
     <row r="23" spans="1:22" ht="96" x14ac:dyDescent="0.2">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
-      <c r="C23" s="17">
+      <c r="C23" s="15">
         <v>16</v>
       </c>
-      <c r="D23" s="17" t="s">
-        <v>68</v>
-      </c>
-      <c r="E23" s="17" t="s">
+      <c r="D23" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="E23" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="F23" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="G23" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="H23" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="I23" s="15" t="s">
+        <v>163</v>
+      </c>
+      <c r="J23" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="F23" s="17" t="s">
-        <v>74</v>
-      </c>
-      <c r="G23" s="17" t="s">
-        <v>75</v>
-      </c>
-      <c r="H23" s="17" t="s">
-        <v>82</v>
-      </c>
-      <c r="I23" s="17" t="s">
-        <v>168</v>
-      </c>
-      <c r="J23" s="17" t="s">
-        <v>83</v>
-      </c>
       <c r="K23" s="13" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="L23" s="1"/>
       <c r="M23" s="1"/>
@@ -2091,32 +2123,32 @@
     <row r="24" spans="1:22" ht="62.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
-      <c r="C24" s="15">
+      <c r="C24" s="14">
         <v>17</v>
       </c>
-      <c r="D24" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="E24" s="15" t="s">
+      <c r="D24" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="E24" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="F24" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="G24" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="H24" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="I24" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="J24" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="F24" s="15" t="s">
-        <v>74</v>
-      </c>
-      <c r="G24" s="15" t="s">
-        <v>75</v>
-      </c>
-      <c r="H24" s="15" t="s">
-        <v>85</v>
-      </c>
-      <c r="I24" s="15" t="s">
-        <v>157</v>
-      </c>
-      <c r="J24" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="K24" s="15" t="s">
-        <v>171</v>
+      <c r="K24" s="14" t="s">
+        <v>166</v>
       </c>
       <c r="L24" s="1"/>
       <c r="M24" s="1"/>
@@ -2130,34 +2162,34 @@
       <c r="U24" s="2"/>
       <c r="V24" s="2"/>
     </row>
-    <row r="25" spans="1:22" ht="64" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:22" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
-      <c r="C25" s="10">
+      <c r="C25" s="25">
         <v>18</v>
       </c>
-      <c r="D25" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="E25" s="10" t="s">
+      <c r="D25" s="25" t="s">
+        <v>67</v>
+      </c>
+      <c r="E25" s="25" t="s">
+        <v>85</v>
+      </c>
+      <c r="F25" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="G25" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="H25" s="25" t="s">
+        <v>86</v>
+      </c>
+      <c r="I25" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="J25" s="25" t="s">
         <v>87</v>
       </c>
-      <c r="F25" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="G25" s="10" t="s">
-        <v>75</v>
-      </c>
-      <c r="H25" s="10" t="s">
-        <v>88</v>
-      </c>
-      <c r="I25" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="J25" s="10" t="s">
-        <v>89</v>
-      </c>
-      <c r="K25" s="10" t="s">
+      <c r="K25" s="25" t="s">
         <v>26</v>
       </c>
       <c r="L25" s="1"/>
@@ -2175,32 +2207,32 @@
     <row r="26" spans="1:22" ht="81.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
-      <c r="C26" s="15">
+      <c r="C26" s="14">
         <v>22</v>
       </c>
-      <c r="D26" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="E26" s="15" t="s">
+      <c r="D26" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="E26" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="F26" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="G26" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="F26" s="15" t="s">
+      <c r="H26" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="I26" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="J26" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="G26" s="15" t="s">
-        <v>92</v>
-      </c>
-      <c r="H26" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="I26" s="15" t="s">
-        <v>157</v>
-      </c>
-      <c r="J26" s="15" t="s">
-        <v>93</v>
-      </c>
-      <c r="K26" s="15" t="s">
-        <v>172</v>
+      <c r="K26" s="14" t="s">
+        <v>167</v>
       </c>
       <c r="L26" s="1"/>
       <c r="M26" s="1"/>
@@ -2214,34 +2246,34 @@
       <c r="U26" s="2"/>
       <c r="V26" s="2"/>
     </row>
-    <row r="27" spans="1:22" ht="80" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:22" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
-      <c r="C27" s="10">
+      <c r="C27" s="25">
         <v>20</v>
       </c>
-      <c r="D27" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="E27" s="10" t="s">
+      <c r="D27" s="25" t="s">
+        <v>67</v>
+      </c>
+      <c r="E27" s="25" t="s">
+        <v>92</v>
+      </c>
+      <c r="F27" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="G27" s="25" t="s">
+        <v>93</v>
+      </c>
+      <c r="H27" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="F27" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="G27" s="10" t="s">
+      <c r="I27" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="J27" s="25" t="s">
         <v>95</v>
       </c>
-      <c r="H27" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="I27" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="J27" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="K27" s="10" t="s">
+      <c r="K27" s="25" t="s">
         <v>26</v>
       </c>
       <c r="L27" s="1"/>
@@ -2256,34 +2288,34 @@
       <c r="U27" s="2"/>
       <c r="V27" s="2"/>
     </row>
-    <row r="28" spans="1:22" ht="64" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:22" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
-      <c r="C28" s="10">
+      <c r="C28" s="25">
         <v>21</v>
       </c>
-      <c r="D28" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="E28" s="10" t="s">
+      <c r="D28" s="25" t="s">
+        <v>67</v>
+      </c>
+      <c r="E28" s="25" t="s">
+        <v>96</v>
+      </c>
+      <c r="F28" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="G28" s="25" t="s">
+        <v>97</v>
+      </c>
+      <c r="H28" s="25" t="s">
         <v>98</v>
       </c>
-      <c r="F28" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="G28" s="10" t="s">
+      <c r="I28" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="J28" s="25" t="s">
         <v>99</v>
       </c>
-      <c r="H28" s="10" t="s">
-        <v>100</v>
-      </c>
-      <c r="I28" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="J28" s="10" t="s">
-        <v>101</v>
-      </c>
-      <c r="K28" s="10" t="s">
+      <c r="K28" s="25" t="s">
         <v>26</v>
       </c>
       <c r="L28" s="1"/>
@@ -2298,34 +2330,34 @@
       <c r="U28" s="2"/>
       <c r="V28" s="2"/>
     </row>
-    <row r="29" spans="1:22" ht="48" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:22" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
-      <c r="C29" s="10">
+      <c r="C29" s="25">
         <v>23</v>
       </c>
-      <c r="D29" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="E29" s="10" t="s">
+      <c r="D29" s="25" t="s">
+        <v>67</v>
+      </c>
+      <c r="E29" s="25" t="s">
+        <v>100</v>
+      </c>
+      <c r="F29" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="G29" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="H29" s="25" t="s">
+        <v>101</v>
+      </c>
+      <c r="I29" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="J29" s="25" t="s">
         <v>102</v>
       </c>
-      <c r="F29" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="G29" s="10" t="s">
-        <v>75</v>
-      </c>
-      <c r="H29" s="10" t="s">
-        <v>103</v>
-      </c>
-      <c r="I29" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="J29" s="10" t="s">
-        <v>104</v>
-      </c>
-      <c r="K29" s="10" t="s">
+      <c r="K29" s="25" t="s">
         <v>26</v>
       </c>
       <c r="L29" s="1"/>
@@ -2340,34 +2372,34 @@
       <c r="U29" s="2"/>
       <c r="V29" s="2"/>
     </row>
-    <row r="30" spans="1:22" ht="96" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:22" ht="96" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
-      <c r="C30" s="10">
+      <c r="C30" s="25">
         <v>24</v>
       </c>
-      <c r="D30" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="E30" s="10" t="s">
+      <c r="D30" s="25" t="s">
+        <v>67</v>
+      </c>
+      <c r="E30" s="25" t="s">
+        <v>103</v>
+      </c>
+      <c r="F30" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="G30" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="H30" s="25" t="s">
         <v>105</v>
       </c>
-      <c r="F30" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="G30" s="10" t="s">
+      <c r="I30" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="J30" s="25" t="s">
         <v>106</v>
       </c>
-      <c r="H30" s="10" t="s">
-        <v>107</v>
-      </c>
-      <c r="I30" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="J30" s="10" t="s">
-        <v>108</v>
-      </c>
-      <c r="K30" s="10" t="s">
+      <c r="K30" s="25" t="s">
         <v>26</v>
       </c>
       <c r="L30" s="1"/>
@@ -2382,32 +2414,32 @@
       <c r="U30" s="2"/>
       <c r="V30" s="2"/>
     </row>
-    <row r="31" spans="1:22" ht="119" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:22" ht="119" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
-      <c r="C31" s="10">
+      <c r="C31" s="25">
         <v>25</v>
       </c>
-      <c r="D31" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="E31" s="10" t="s">
-        <v>109</v>
+      <c r="D31" s="25" t="s">
+        <v>67</v>
+      </c>
+      <c r="E31" s="25" t="s">
+        <v>107</v>
       </c>
       <c r="F31" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="G31" s="10" t="s">
-        <v>106</v>
-      </c>
-      <c r="H31" s="10"/>
-      <c r="I31" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="G31" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="H31" s="25"/>
+      <c r="I31" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="J31" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="K31" s="10" t="s">
+      <c r="J31" s="25" t="s">
+        <v>108</v>
+      </c>
+      <c r="K31" s="25" t="s">
         <v>26</v>
       </c>
       <c r="L31" s="1"/>
@@ -2429,26 +2461,26 @@
         <v>26</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E32" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="F32" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="G32" s="9" t="s">
         <v>111</v>
-      </c>
-      <c r="F32" s="9" t="s">
-        <v>112</v>
-      </c>
-      <c r="G32" s="9" t="s">
-        <v>113</v>
       </c>
       <c r="H32" s="9"/>
       <c r="I32" s="9" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="J32" s="9" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="K32" s="8" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="L32" s="1"/>
       <c r="M32" s="1"/>
@@ -2462,34 +2494,34 @@
       <c r="U32" s="2"/>
       <c r="V32" s="2"/>
     </row>
-    <row r="33" spans="1:22" ht="64" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:22" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
-      <c r="C33" s="10">
+      <c r="C33" s="25">
         <v>27</v>
       </c>
-      <c r="D33" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="E33" s="10" t="s">
+      <c r="D33" s="25" t="s">
+        <v>67</v>
+      </c>
+      <c r="E33" s="25" t="s">
+        <v>113</v>
+      </c>
+      <c r="F33" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="G33" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="H33" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="I33" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="J33" s="25" t="s">
         <v>115</v>
       </c>
-      <c r="F33" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="G33" s="10" t="s">
-        <v>75</v>
-      </c>
-      <c r="H33" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="I33" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="J33" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="K33" s="10"/>
+      <c r="K33" s="25"/>
       <c r="L33" s="1"/>
       <c r="M33" s="1"/>
       <c r="N33" s="1"/>
@@ -2509,28 +2541,28 @@
         <v>28</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E34" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="F34" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="G34" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="H34" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="F34" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="G34" s="9" t="s">
+      <c r="I34" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="J34" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="H34" s="9" t="s">
-        <v>120</v>
-      </c>
-      <c r="I34" s="9" t="s">
-        <v>157</v>
-      </c>
-      <c r="J34" s="9" t="s">
-        <v>121</v>
-      </c>
       <c r="K34" s="8" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="L34" s="1"/>
       <c r="M34" s="1"/>
@@ -2544,35 +2576,35 @@
       <c r="U34" s="2"/>
       <c r="V34" s="2"/>
     </row>
-    <row r="35" spans="1:22" ht="48" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:22" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
-      <c r="C35" s="10">
+      <c r="C35" s="25">
         <v>29</v>
       </c>
-      <c r="D35" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="E35" s="10" t="s">
+      <c r="D35" s="25" t="s">
+        <v>67</v>
+      </c>
+      <c r="E35" s="25" t="s">
+        <v>120</v>
+      </c>
+      <c r="F35" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="G35" s="25" t="s">
         <v>122</v>
       </c>
-      <c r="F35" s="10" t="s">
+      <c r="H35" s="25" t="s">
         <v>123</v>
       </c>
-      <c r="G35" s="10" t="s">
+      <c r="I35" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="J35" s="25" t="s">
         <v>124</v>
       </c>
-      <c r="H35" s="10" t="s">
-        <v>125</v>
-      </c>
-      <c r="I35" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="J35" s="10" t="s">
-        <v>126</v>
-      </c>
-      <c r="K35" s="10" t="s">
-        <v>175</v>
+      <c r="K35" s="25" t="s">
+        <v>170</v>
       </c>
       <c r="L35" s="1"/>
       <c r="M35" s="1"/>
@@ -2593,28 +2625,28 @@
         <v>30</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E36" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="F36" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="G36" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="F36" s="9" t="s">
+      <c r="H36" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="G36" s="9" t="s">
+      <c r="I36" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="J36" s="9" t="s">
         <v>129</v>
       </c>
-      <c r="H36" s="9" t="s">
-        <v>130</v>
-      </c>
-      <c r="I36" s="9" t="s">
-        <v>157</v>
-      </c>
-      <c r="J36" s="9" t="s">
-        <v>131</v>
-      </c>
       <c r="K36" s="9" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="L36" s="1"/>
       <c r="M36" s="1"/>
@@ -2635,28 +2667,28 @@
         <v>31</v>
       </c>
       <c r="D37" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E37" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="F37" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="G37" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="H37" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="I37" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="J37" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="F37" s="9" t="s">
-        <v>128</v>
-      </c>
-      <c r="G37" s="9" t="s">
-        <v>129</v>
-      </c>
-      <c r="H37" s="9" t="s">
-        <v>133</v>
-      </c>
-      <c r="I37" s="9" t="s">
-        <v>157</v>
-      </c>
-      <c r="J37" s="9" t="s">
-        <v>134</v>
-      </c>
       <c r="K37" s="9" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="L37" s="1"/>
       <c r="M37" s="1"/>
@@ -2670,35 +2702,35 @@
       <c r="U37" s="2"/>
       <c r="V37" s="2"/>
     </row>
-    <row r="38" spans="1:22" ht="48" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:22" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
-      <c r="C38" s="10">
+      <c r="C38" s="25">
         <v>32</v>
       </c>
-      <c r="D38" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="E38" s="10" t="s">
+      <c r="D38" s="25" t="s">
+        <v>67</v>
+      </c>
+      <c r="E38" s="25" t="s">
+        <v>133</v>
+      </c>
+      <c r="F38" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="G38" s="25" t="s">
+        <v>134</v>
+      </c>
+      <c r="H38" s="25" t="s">
         <v>135</v>
       </c>
-      <c r="F38" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="G38" s="10" t="s">
+      <c r="I38" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="J38" s="25" t="s">
         <v>136</v>
       </c>
-      <c r="H38" s="10" t="s">
-        <v>137</v>
-      </c>
-      <c r="I38" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="J38" s="10" t="s">
-        <v>138</v>
-      </c>
-      <c r="K38" s="11" t="s">
-        <v>178</v>
+      <c r="K38" s="27" t="s">
+        <v>173</v>
       </c>
       <c r="L38" s="1"/>
       <c r="M38" s="1"/>
@@ -2712,35 +2744,35 @@
       <c r="U38" s="2"/>
       <c r="V38" s="2"/>
     </row>
-    <row r="39" spans="1:22" ht="96" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:22" ht="96" hidden="1" x14ac:dyDescent="0.2">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
-      <c r="C39" s="18">
+      <c r="C39" s="25">
         <v>33</v>
       </c>
-      <c r="D39" s="18" t="s">
-        <v>68</v>
-      </c>
-      <c r="E39" s="18" t="s">
+      <c r="D39" s="25" t="s">
+        <v>67</v>
+      </c>
+      <c r="E39" s="25" t="s">
+        <v>137</v>
+      </c>
+      <c r="F39" s="16" t="s">
+        <v>138</v>
+      </c>
+      <c r="G39" s="25" t="s">
         <v>139</v>
       </c>
-      <c r="F39" s="18" t="s">
+      <c r="H39" s="25" t="s">
         <v>140</v>
       </c>
-      <c r="G39" s="18" t="s">
+      <c r="I39" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="J39" s="25" t="s">
         <v>141</v>
       </c>
-      <c r="H39" s="18" t="s">
-        <v>142</v>
-      </c>
-      <c r="I39" s="18" t="s">
-        <v>26</v>
-      </c>
-      <c r="J39" s="18" t="s">
-        <v>143</v>
-      </c>
-      <c r="K39" s="18" t="s">
-        <v>179</v>
+      <c r="K39" s="25" t="s">
+        <v>174</v>
       </c>
       <c r="L39" s="1"/>
       <c r="M39" s="1"/>
@@ -2761,28 +2793,28 @@
         <v>34</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E40" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="F40" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="G40" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="H40" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="F40" s="9" t="s">
-        <v>140</v>
-      </c>
-      <c r="G40" s="9" t="s">
+      <c r="I40" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="J40" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="H40" s="9" t="s">
-        <v>146</v>
-      </c>
-      <c r="I40" s="9" t="s">
-        <v>157</v>
-      </c>
-      <c r="J40" s="9" t="s">
-        <v>147</v>
-      </c>
       <c r="K40" s="9" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="L40" s="1"/>
       <c r="M40" s="1"/>
@@ -2803,28 +2835,28 @@
         <v>35</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E41" s="9" t="s">
+        <v>146</v>
+      </c>
+      <c r="F41" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="G41" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="H41" s="9" t="s">
         <v>148</v>
       </c>
-      <c r="F41" s="9" t="s">
-        <v>140</v>
-      </c>
-      <c r="G41" s="9" t="s">
+      <c r="I41" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="J41" s="9" t="s">
         <v>149</v>
       </c>
-      <c r="H41" s="9" t="s">
-        <v>150</v>
-      </c>
-      <c r="I41" s="9" t="s">
-        <v>157</v>
-      </c>
-      <c r="J41" s="9" t="s">
-        <v>151</v>
-      </c>
       <c r="K41" s="8" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="L41" s="1"/>
       <c r="M41" s="1"/>
@@ -2845,28 +2877,28 @@
         <v>36</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E42" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="F42" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="G42" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="F42" s="9" t="s">
+      <c r="H42" s="9" t="s">
         <v>153</v>
       </c>
-      <c r="G42" s="9" t="s">
+      <c r="I42" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="J42" s="9" t="s">
         <v>154</v>
       </c>
-      <c r="H42" s="9" t="s">
-        <v>155</v>
-      </c>
-      <c r="I42" s="9" t="s">
-        <v>157</v>
-      </c>
-      <c r="J42" s="9" t="s">
-        <v>156</v>
-      </c>
       <c r="K42" s="8" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="L42" s="1"/>
       <c r="M42" s="1"/>
@@ -25873,10 +25905,15 @@
       <c r="V1000" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A7:J42" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A7:J42">
-      <sortCondition ref="D7:D42"/>
-    </sortState>
+  <autoFilter ref="A7:K42" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="8">
+      <filters>
+        <filter val="Cumple parcialmente."/>
+        <filter val="Cumple, Parcialmente"/>
+        <filter val="En progreso."/>
+        <filter val="No Cumple."/>
+      </filters>
+    </filterColumn>
   </autoFilter>
   <mergeCells count="5">
     <mergeCell ref="D2:I2"/>

</xml_diff>